<commit_message>
Implement backend Sprint 1-2: auth/RBAC, categories, suppliers, products, employees, import lots
- FastAPI layered app (router/service/repository) wired to PostgreSQL via psycopg3 pool
- JWT access+refresh auth with rotation, bcrypt password hashing, 3-role RBAC dependency
- CRUD APIs: categories, suppliers, products+variants (search/filter/sort/pagination),
  staff management (create/update/lock/unlock), import lots (restocks inventory via the
  restock_from_import() stored procedure)
- Cross-cutting: audit log on every mutation, soft-delete, Redis cache with invalidation,
  Excel product import with per-row error isolation
- database/seed.sql with demo admin/staff/customer accounts and sample catalog data
- docs/TBookStore.postman_collection.json for manual Postman testing
- Verified end-to-end against dockerized postgres+redis+api (all endpoints, RBAC, cache,
  audit log, stock restock confirmed working)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TBookStore_MasterPlan_VER2.xlsx
+++ b/TBookStore_MasterPlan_VER2.xlsx
@@ -62,7 +62,7 @@
     <t xml:space="preserve">Kiến trúc</t>
   </si>
   <si>
-    <t xml:space="preserve">Khởi tạo project .NET 8 Web API, cấu trúc layer Controller/Service/Repository</t>
+    <t xml:space="preserve">Khởi tạo project FastAPI (Python 3.12), cấu trúc layer Router/Service/Repository</t>
   </si>
   <si>
     <t xml:space="preserve">Must</t>
@@ -83,7 +83,7 @@
     <t xml:space="preserve">Database</t>
   </si>
   <si>
-    <t xml:space="preserve">Chuyển schema MySQL → SQL Server (ENUM→CHECK, AUTO_INCREMENT→IDENTITY)</t>
+    <t xml:space="preserve">Chuyển schema MySQL → PostgreSQL (giữ ENUM type, AUTO_INCREMENT→GENERATED ALWAYS AS IDENTITY)</t>
   </si>
   <si>
     <t xml:space="preserve">1d</t>
@@ -95,7 +95,7 @@
     <t xml:space="preserve">Giữ nguyên tên bảng/cột để đỡ đổi logic</t>
   </si>
   <si>
-    <t xml:space="preserve">Cấu hình Dapper + connection factory + stored procedure mẫu</t>
+    <t xml:space="preserve">Cấu hình psycopg 3 + connection pool + stored procedure mẫu</t>
   </si>
   <si>
     <t xml:space="preserve">Auth</t>
@@ -143,7 +143,7 @@
     <t xml:space="preserve">Swagger/OpenAPI setup</t>
   </si>
   <si>
-    <t xml:space="preserve">Docker Compose khung sườn (api + sqlserver)</t>
+    <t xml:space="preserve">Docker Compose khung sườn (api + postgres)</t>
   </si>
   <si>
     <t xml:space="preserve">Should</t>
@@ -404,7 +404,7 @@
     <t xml:space="preserve">Xuất file</t>
   </si>
   <si>
-    <t xml:space="preserve">API xuất PDF hóa đơn/báo cáo bằng QuestPDF</t>
+    <t xml:space="preserve">API xuất PDF hóa đơn/báo cáo bằng ReportLab</t>
   </si>
   <si>
     <t xml:space="preserve">views/*/print.ejs</t>
@@ -416,7 +416,7 @@
     <t xml:space="preserve">Job nền</t>
   </si>
   <si>
-    <t xml:space="preserve">Hàng đợi tác vụ (Hangfire) cho gửi mail &amp; xuất báo cáo lớn</t>
+    <t xml:space="preserve">Hàng đợi tác vụ (Celery) cho gửi mail &amp; xuất báo cáo lớn</t>
   </si>
   <si>
     <t xml:space="preserve">Chất lượng</t>
@@ -437,7 +437,7 @@
     <t xml:space="preserve">middlewares/rateLimit.middleware.js</t>
   </si>
   <si>
-    <t xml:space="preserve">Health check endpoint + logging có cấu trúc (Serilog)</t>
+    <t xml:space="preserve">Health check endpoint + logging có cấu trúc (structlog)</t>
   </si>
   <si>
     <t xml:space="preserve">Triển khai</t>
@@ -527,13 +527,13 @@
     <t xml:space="preserve">Chỉ bán online (không bán tại quầy/POS)</t>
   </si>
   <si>
-    <t xml:space="preserve">Tách rời Backend (ASP.NET Core Web API + Dapper + SQL Server) và Frontend (AngularJS SPA gọi API qua JWT), khác với project cũ vốn dùng EJS render phía server</t>
+    <t xml:space="preserve">Tách rời Backend (FastAPI + psycopg 3 + PostgreSQL) và Frontend (AngularJS SPA gọi API qua JWT), khác với project cũ vốn dùng EJS render phía server</t>
   </si>
   <si>
     <t xml:space="preserve">Stack</t>
   </si>
   <si>
-    <t xml:space="preserve">.NET 8 (ASP.NET Core) + Dapper + SQL Server + AngularJS + Redis + Docker Compose</t>
+    <t xml:space="preserve">FastAPI (Python 3.12) + psycopg 3 + PostgreSQL + AngularJS + Redis + Docker Compose</t>
   </si>
   <si>
     <t xml:space="preserve">Tham khảo</t>

</xml_diff>